<commit_message>
El tope de 10 aplica desde la próxima corrida, no retroactivamente
Los reportes ya emitidos (24, 25 y 26 de agosto) conservan su formato original.
El tope rige para las búsquedas siguientes, así que el PR deja de tocar los
archivos de resultados y se limita al generador, la skill y los prompts.
</commit_message>
<xml_diff>
--- a/resultados/Fiscalizacion_Web_DM_agujas-hipodermicas_24-08-2026.xlsx
+++ b/resultados/Fiscalizacion_Web_DM_agujas-hipodermicas_24-08-2026.xlsx
@@ -8,11 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Hallazgos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Anexo — sobre el tope" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Búsquedas Marketplace" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Búsquedas Marketplace" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hallazgos'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hallazgos'!$A$1:$K$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,10 +40,6 @@
     <font>
       <b val="1"/>
       <color rgb="001E6B1E"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -106,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -126,7 +121,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -999,230 +993,307 @@
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodérmica caja x 100 unidades Cranberry</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>https://deltamed.cl/tienda/producto/aguja-hipodermica-caja-x-100-unidades-cranberry/</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodérmica caja x 100 unidades Cranberry</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Deltamed</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>CRANBERRY</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>DM 397/15</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>La publicación no especifica calibre. Se cita DM 397/15 por ser el de mayor cobertura de la marca (19G, 21G, 23G, 25G, 27G). Verificar calibre concreto si se fiscaliza.</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Agujas Hipodérmicas Cranberry caja 100 unidades</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>https://klinetix.cl/products/agujas-hipodermicas-cranberry</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Agujas Hipodérmicas Cranberry</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Klinetix</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>CRANBERRY</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>DM 397/15</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Calibre no especificado en la publicación. Klinetix además tiene marca propia registrada (DM 656/25).</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodérmica 24G x 1" 100 unidades Nipro</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vicamat.cl/aguja-hipodermica-24g-x-1-100-und-nipro</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodermica 24G x 1 100 Und - Nipro</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Vicamat</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>NIPRO</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>DM/10AG/0175/09</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>CORRECCIÓN respecto del reporte anterior, que citaba DM 630/24: ese registro no incluye 24G. El calibre 24G x 1 sí está en DM/10AG/0175/09. Solo dos registros del listado cubren 24G.</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Caja Aguja Hipodérmica 27G x 1/2 - 100 unidades Nipro Flomax</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>https://medcare.cl/products/caja-aguja-hipodermica-27g-x-1-2-100-unidades</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Caja Aguja Hipodérmica 27G x 1/2 -100 Unidades</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Medcare</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>NIPRO</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>DM 630/24</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>El título es genérico pero la descripción declara Nipro Flomax. Calibre 27G x 1/2 verificado en DM 630/24. Precio $8.990.</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodérmica 19G x 1 1/2 Medicaltek caja 100 unidades</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.osm.cl/product-page/aguja-hipodermica-19g-x-1-1-2-medicaltek-caja-100-unidades</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Aguja Hipodermica 19G x 1 1/2 Medicaltek caja 100 unidades</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>OSM Ltda</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>MEDICALTEK</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>DM 412/15</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Calibre 19G x 1 1/2 verificado en el registro. Titular Medicaltek Chile S.A. Precio $4.740.</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Agujas hipodérmicas Cranberry caja 100 unidades</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>https://nexodental.cl/product/agujas-hipodermicas-100-unidades-cranberry/</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>agujas hipodérmicas Cranberry | Caja 100 unidades</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Nexo Dental</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>CRANBERRY</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>DM 397/15</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>REGISTRADO</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Calibre no especificado. Oferente del rubro dental.</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
+  <autoFilter ref="A1:K17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Nombre de DM ofertado</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Oferente</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Clasificación</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Aguja Hipodérmica caja x 100 unidades Cranberry</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>https://deltamed.cl/tienda/producto/aguja-hipodermica-caja-x-100-unidades-cranberry/</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Deltamed</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>La publicación no especifica calibre. Se cita DM 397/15 por ser el de mayor cobertura de la marca (19G, 21G, 23G, 25G, 27G). Verificar calibre concreto si se fiscaliza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Agujas Hipodérmicas Cranberry caja 100 unidades</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>https://klinetix.cl/products/agujas-hipodermicas-cranberry</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Klinetix</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Calibre no especificado en la publicación. Klinetix además tiene marca propia registrada (DM 656/25).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Aguja Hipodérmica 24G x 1" 100 unidades Nipro</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.vicamat.cl/aguja-hipodermica-24g-x-1-100-und-nipro</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Vicamat</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>CORRECCIÓN respecto del reporte anterior, que citaba DM 630/24: ese registro no incluye 24G. El calibre 24G x 1 sí está en DM/10AG/0175/09. Solo dos registros del listado cubren 24G.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Caja Aguja Hipodérmica 27G x 1/2 - 100 unidades Nipro Flomax</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>https://medcare.cl/products/caja-aguja-hipodermica-27g-x-1-2-100-unidades</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Medcare</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>El título es genérico pero la descripción declara Nipro Flomax. Calibre 27G x 1/2 verificado en DM 630/24. Precio $8.990.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Aguja Hipodérmica 19G x 1 1/2 Medicaltek caja 100 unidades</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.osm.cl/product-page/aguja-hipodermica-19g-x-1-1-2-medicaltek-caja-100-unidades</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>OSM Ltda</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Calibre 19G x 1 1/2 verificado en el registro. Titular Medicaltek Chile S.A. Precio $4.740.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Agujas hipodérmicas Cranberry caja 100 unidades</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>https://nexodental.cl/product/agujas-hipodermicas-100-unidades-cranberry/</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Nexo Dental</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>REGISTRADO</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Calibre no especificado. Oferente del rubro dental.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Estas 6 ofertas se detectaron en la misma búsqueda pero quedaron fuera del reporte por el tope de 10 hallazgos. NO requieren revisión esta semana. Al no quedar registradas como evaluadas, vuelven a considerarse en la próxima corrida de la categoría.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>